<commit_message>
Revisione: quota del vecchio gestionale dopo l'annullamento, righe vuote del foglio, link solo agli utenti attivi, limiti sulle pagine della password
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkHEzxKYLrW47WYQvDfkoT
</commit_message>
<xml_diff>
--- a/tests/fixtures/soci-buoni.xlsx
+++ b/tests/fixtures/soci-buoni.xlsx
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="J4" s="15" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
@@ -1521,7 +1521,7 @@
       <c r="I5" s="12" t="n"/>
       <c r="J5" s="15" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="K5" s="11" t="n"/>
@@ -1620,7 +1620,11 @@
       <c r="H7" s="11" t="n"/>
       <c r="I7" s="12" t="n"/>
       <c r="J7" s="15" t="n"/>
-      <c r="K7" s="11" t="n"/>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="L7" s="15" t="n"/>
       <c r="M7" s="11" t="n"/>
       <c r="N7" s="12" t="n"/>
@@ -1640,7 +1644,11 @@
       <c r="H8" s="11" t="n"/>
       <c r="I8" s="12" t="n"/>
       <c r="J8" s="15" t="n"/>
-      <c r="K8" s="11" t="n"/>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="L8" s="15" t="n"/>
       <c r="M8" s="11" t="n"/>
       <c r="N8" s="12" t="n"/>
@@ -1660,7 +1668,11 @@
       <c r="H9" s="11" t="n"/>
       <c r="I9" s="12" t="n"/>
       <c r="J9" s="15" t="n"/>
-      <c r="K9" s="11" t="n"/>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="L9" s="15" t="n"/>
       <c r="M9" s="11" t="n"/>
       <c r="N9" s="12" t="n"/>
@@ -1680,7 +1692,11 @@
       <c r="H10" s="11" t="n"/>
       <c r="I10" s="12" t="n"/>
       <c r="J10" s="15" t="n"/>
-      <c r="K10" s="11" t="n"/>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="11" t="n"/>
       <c r="N10" s="12" t="n"/>
@@ -1700,7 +1716,11 @@
       <c r="H11" s="11" t="n"/>
       <c r="I11" s="12" t="n"/>
       <c r="J11" s="15" t="n"/>
-      <c r="K11" s="11" t="n"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="L11" s="15" t="n"/>
       <c r="M11" s="11" t="n"/>
       <c r="N11" s="12" t="n"/>
@@ -1710,7 +1730,11 @@
       <c r="R11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   </t>
+        </is>
+      </c>
       <c r="B12" s="11" t="n"/>
       <c r="C12" s="12" t="n"/>
       <c r="D12" s="11" t="n"/>

</xml_diff>